<commit_message>
Sheet snapshots of 29 September 2026, Lasri capitalised across the data, Excel lock file removed
The .xlsx files re-downloaded on 29 September (Janus Statistics, Atirha Cities, soldier counts, oil and gas, population growth, production, skyscrapers, FLLA rankings) and the data files rebuilt from them; lasri becomes Lasri in countries.json, the wiki dump copy, the FLLA data and the simulation notes; the stray ~$Population Growth(2).xlsx lock file is deleted.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/.xlsx files/Atirha Cities.xlsx
+++ b/.xlsx files/Atirha Cities.xlsx
@@ -14,7 +14,7 @@
     <sheet state="visible" name="Grazail" sheetId="9" r:id="rId13"/>
     <sheet state="visible" name="Guise" sheetId="10" r:id="rId14"/>
     <sheet state="visible" name="Laselteh" sheetId="11" r:id="rId15"/>
-    <sheet state="visible" name="lasri" sheetId="12" r:id="rId16"/>
+    <sheet state="visible" name="Lasri" sheetId="12" r:id="rId16"/>
     <sheet state="visible" name="Metndria" sheetId="13" r:id="rId17"/>
     <sheet state="visible" name="New Misos" sheetId="14" r:id="rId18"/>
     <sheet state="visible" name="Peka" sheetId="15" r:id="rId19"/>
@@ -1204,7 +1204,7 @@
       <tableStyleElement dxfId="3" type="secondRowStripe"/>
       <tableStyleElement dxfId="4" size="0" type="wholeTable"/>
     </tableStyle>
-    <tableStyle count="4" pivot="0" name="lasri-style">
+    <tableStyle count="4" pivot="0" name="Lasri-style">
       <tableStyleElement dxfId="1" type="headerRow"/>
       <tableStyleElement dxfId="2" type="firstRowStripe"/>
       <tableStyleElement dxfId="3" type="secondRowStripe"/>
@@ -1389,7 +1389,7 @@
 </file>
 
 <file path=xl/tables/table12.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:F3" displayName="lasri" name="lasri" id="12">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:F3" displayName="Lasri" name="Lasri" id="12">
   <tableColumns count="6">
     <tableColumn name="City Name" id="1"/>
     <tableColumn name="Population" id="2"/>
@@ -1398,7 +1398,7 @@
     <tableColumn name="Column 5" id="5"/>
     <tableColumn name="Column 6" id="6"/>
   </tableColumns>
-  <tableStyleInfo name="lasri-style" showColumnStripes="0" showFirstColumn="1" showLastColumn="1" showRowStripes="1"/>
+  <tableStyleInfo name="Lasri-style" showColumnStripes="0" showFirstColumn="1" showLastColumn="1" showRowStripes="1"/>
 </table>
 </file>
 

</xml_diff>